<commit_message>
Renombrar PIV como poblacion inscrita y validada
</commit_message>
<xml_diff>
--- a/output/cobertura_mamografia_rm_2025.xlsx
+++ b/output/cobertura_mamografia_rm_2025.xlsx
@@ -9,14 +9,14 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="comuna_dic" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="establecimiento_control" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="denominador_piv" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="denominador" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="control" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metodologia" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'comuna_dic'!$A$1:$H$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'establecimiento_control'!$A$1:$Z$262</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'denominador_piv'!$A$1:$P$294</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'denominador'!$A$1:$P$294</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'control'!$A$1:$N$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'metodologia'!$A$1:$B$10</definedName>
   </definedNames>
@@ -455,7 +455,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
@@ -488,7 +488,7 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>denominador_piv_mujeres_50_69</t>
+          <t>denominador_poblacion_inscrita_validada_mujeres_50_69</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
@@ -2088,11 +2088,11 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="45" customWidth="1" min="15" max="15"/>
-    <col width="31" customWidth="1" min="16" max="16"/>
+    <col width="45" customWidth="1" min="16" max="16"/>
     <col width="21" customWidth="1" min="17" max="17"/>
     <col width="45" customWidth="1" min="18" max="18"/>
     <col width="45" customWidth="1" min="19" max="19"/>
@@ -2163,27 +2163,27 @@
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>servicio_salud_piv</t>
+          <t>servicio_salud_denominador</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>dependencia_piv</t>
+          <t>dependencia_denominador</t>
         </is>
       </c>
       <c r="N1" s="2" t="inlineStr">
         <is>
-          <t>comuna_piv</t>
+          <t>comuna_denominador</t>
         </is>
       </c>
       <c r="O1" s="2" t="inlineStr">
         <is>
-          <t>establecimiento_piv</t>
+          <t>establecimiento_denominador</t>
         </is>
       </c>
       <c r="P1" s="2" t="inlineStr">
         <is>
-          <t>denominador_piv_mujeres_50_69</t>
+          <t>denominador_poblacion_inscrita_validada_mujeres_50_69</t>
         </is>
       </c>
       <c r="Q1" s="2" t="inlineStr">
@@ -6102,7 +6102,7 @@
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>Sin denominador PIV directo; no usar como cobertura establecimiento</t>
+          <t>Sin población inscrita y validada directa; no usar como cobertura establecimiento</t>
         </is>
       </c>
     </row>
@@ -6177,7 +6177,7 @@
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>Sin denominador PIV directo; no usar como cobertura establecimiento</t>
+          <t>Sin población inscrita y validada directa; no usar como cobertura establecimiento</t>
         </is>
       </c>
     </row>
@@ -8687,7 +8687,7 @@
       </c>
       <c r="Z68" t="inlineStr">
         <is>
-          <t>Sin denominador PIV directo; no usar como cobertura establecimiento</t>
+          <t>Sin población inscrita y validada directa; no usar como cobertura establecimiento</t>
         </is>
       </c>
     </row>
@@ -9055,7 +9055,7 @@
       </c>
       <c r="Z72" t="inlineStr">
         <is>
-          <t>Sin denominador PIV directo; no usar como cobertura establecimiento</t>
+          <t>Sin población inscrita y validada directa; no usar como cobertura establecimiento</t>
         </is>
       </c>
     </row>
@@ -24337,7 +24337,7 @@
       </c>
       <c r="Z230" t="inlineStr">
         <is>
-          <t>Sin denominador PIV directo; no usar como cobertura establecimiento</t>
+          <t>Sin población inscrita y validada directa; no usar como cobertura establecimiento</t>
         </is>
       </c>
     </row>
@@ -27444,12 +27444,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
@@ -27469,32 +27469,32 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>IdEstablecimiento_piv_original</t>
+          <t>IdEstablecimiento_denominador_original</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>servicio_salud_piv</t>
+          <t>servicio_salud_denominador</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>dependencia_piv</t>
+          <t>dependencia_denominador</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>comuna_piv</t>
+          <t>comuna_denominador</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>establecimiento_piv</t>
+          <t>establecimiento_denominador</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>denominador_piv_mujeres_50_69</t>
+          <t>denominador_poblacion_inscrita_validada_mujeres_50_69</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
@@ -49868,13 +49868,13 @@
   <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
@@ -49917,7 +49917,7 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>denominador_piv_mujeres_50_69</t>
+          <t>denominador_poblacion_inscrita_validada_mujeres_50_69</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
@@ -49959,7 +49959,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REM con numerador P12 sin PIV directa</t>
+          <t>REM con numerador P12 sin población inscrita y validada directa</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -50008,7 +50008,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REM con numerador P12 sin PIV directa</t>
+          <t>REM con numerador P12 sin población inscrita y validada directa</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -50057,7 +50057,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REM con numerador P12 sin PIV directa</t>
+          <t>REM con numerador P12 sin población inscrita y validada directa</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -50106,7 +50106,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REM con numerador P12 sin PIV directa</t>
+          <t>REM con numerador P12 sin población inscrita y validada directa</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -50160,7 +50160,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>REM con numerador P12 sin PIV directa</t>
+          <t>REM con numerador P12 sin población inscrita y validada directa</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -50226,7 +50226,7 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -50286,14 +50286,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PIV mujeres 50-69, inscritos 2024, base de pago 2025</t>
+          <t>Población inscrita y validada mujeres 50-69, inscritos 2024, base de pago 2025</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>alias_piv_aplicado</t>
+          <t>alias_denominador_aplicado</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -50322,7 +50322,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>numerador_mujeres_50_69 / denominador_piv_mujeres_50_69 * 100</t>
+          <t>numerador_mujeres_50_69 / denominador_poblacion_inscrita_validada_mujeres_50_69 * 100</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion datos REM 2026-07-06 09:21 (orquestador)
</commit_message>
<xml_diff>
--- a/output/cobertura_mamografia_rm_2025.xlsx
+++ b/output/cobertura_mamografia_rm_2025.xlsx
@@ -27,16 +27,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -56,7 +53,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -64,22 +61,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -461,42 +449,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ano</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>IdRegion</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>IdComuna</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>numerador_mujeres_50_69</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>denominador_poblacion_inscrita_validada_mujeres_50_69</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>comuna_master</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>cobertura_mamografia_pct</t>
         </is>
@@ -2106,132 +2094,132 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Ano</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>IdRegion</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>IdServicio</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>IdComuna</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>IdEstablecimiento</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>50_54</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>55_59</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>60_64</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>65_69</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>numerador_mujeres_50_69</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>servicio_salud_denominador</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>dependencia_denominador</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>comuna_denominador</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>establecimiento_denominador</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>denominador_poblacion_inscrita_validada_mujeres_50_69</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>codigo_madre_master</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>servicio_salud_master</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>tipo_establecimiento_master</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>establecimiento_master</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>dependencia_master</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>comuna_master</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>estado_funcionamiento_master</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>denominador_disponible</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>cobertura_mamografia_pct</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>advertencia_cobertura_establecimiento</t>
         </is>
@@ -27462,82 +27450,82 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>IdEstablecimiento</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>IdEstablecimiento_denominador_original</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>servicio_salud_denominador</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>dependencia_denominador</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>comuna_denominador</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>establecimiento_denominador</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>denominador_poblacion_inscrita_validada_mujeres_50_69</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>codigo_madre_master</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>IdServicio_master</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>servicio_salud_master</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>tipo_establecimiento_master</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>establecimiento_master</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>dependencia_master</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>IdComuna_master</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>comuna_master</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>estado_funcionamiento_master</t>
         </is>
@@ -27579,7 +27567,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -27654,7 +27642,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -27729,7 +27717,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -27804,7 +27792,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -27879,7 +27867,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -27954,7 +27942,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -28029,7 +28017,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -28104,7 +28092,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -28179,7 +28167,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -28254,7 +28242,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -28329,7 +28317,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -28404,7 +28392,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -28479,7 +28467,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -28554,7 +28542,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -28629,7 +28617,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -28704,7 +28692,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -28779,7 +28767,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -28854,7 +28842,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -28929,7 +28917,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -29004,7 +28992,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -29079,7 +29067,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -29154,7 +29142,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -29229,7 +29217,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -29304,7 +29292,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -29379,7 +29367,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -29454,7 +29442,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -29529,7 +29517,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -29604,7 +29592,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -29679,7 +29667,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -29754,7 +29742,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -29829,7 +29817,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -29904,7 +29892,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -29984,7 +29972,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -30064,7 +30052,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -30144,7 +30132,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -30224,7 +30212,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -30304,7 +30292,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -30384,7 +30372,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -30464,7 +30452,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -44309,7 +44297,7 @@
       </c>
       <c r="K222" t="inlineStr">
         <is>
-          <t>Hospital de Campaña</t>
+          <t>Dispositivo Incorporado por Crisis Sanitaria</t>
         </is>
       </c>
       <c r="L222" t="inlineStr">
@@ -48164,7 +48152,7 @@
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
@@ -48484,7 +48472,7 @@
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J277" t="inlineStr">
@@ -49044,7 +49032,7 @@
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
@@ -49124,7 +49112,7 @@
       </c>
       <c r="I285" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J285" t="inlineStr">
@@ -49279,7 +49267,7 @@
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J287" t="inlineStr">
@@ -49509,7 +49497,7 @@
       </c>
       <c r="I290" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J290" t="inlineStr">
@@ -49739,7 +49727,7 @@
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>09</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
@@ -49885,72 +49873,72 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>tipo_control</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>IdServicio</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>IdComuna</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>IdEstablecimiento</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>numerador_mujeres_50_69</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>denominador_poblacion_inscrita_validada_mujeres_50_69</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>cobertura_mamografia_pct</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>codigo_madre_master</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>servicio_salud_master</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>comuna_master</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>establecimiento_master</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>tipo_establecimiento_master</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>estado_funcionamiento_master</t>
         </is>
@@ -50231,12 +50219,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>valor</t>
         </is>

</xml_diff>